<commit_message>
Harvest crystal function fixed. Began on crystal screen upload function.
</commit_message>
<xml_diff>
--- a/CrystalDex_Library.xlsx
+++ b/CrystalDex_Library.xlsx
@@ -53,7 +53,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +64,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9D18E"/>
+        <bgColor rgb="00A9D18E"/>
       </patternFill>
     </fill>
   </fills>
@@ -214,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -240,6 +246,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21417,11 +21429,15 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B8" s="3">
-        <f>_xlfn.TEXTJOIN("",FALSE,$H$1," mg/mL")</f>
-        <v/>
-      </c>
-      <c r="C8" s="11" t="n"/>
+      <c r="B8" s="21">
+        <f>_xlfn.TEXTJOIN("",FALSE,$H$1," mg/mL")</f>
+        <v/>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>1TEL_DARPin_Crystal_Screen_A1_top_left_06-19-2025_06-19-2025_harvested</t>
+        </is>
+      </c>
       <c r="D8" s="3">
         <f>_xlfn.TEXTJOIN("",FALSE,$H$1," mg/mL")</f>
         <v/>
@@ -21599,9 +21615,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Days to 1st Crystal:</t>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Days to 1st Crystal:</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -21793,9 +21814,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Size of largest Crystal:</t>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Size of largest Crystal:</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>281x142 um</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -21987,9 +22013,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Number of harvestable crystals:</t>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Number of harvestable crystals:</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -22181,9 +22212,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Shape:</t>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Shape:</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>Fake</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -22375,9 +22411,14 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Contaminants:</t>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Contaminants:</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>Possible salt crystals: False, precipitation: False, microcrystals: False, glassy protein or artifacts: False</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -22569,12 +22610,17 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Notes:</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n"/>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">None, just a test! Ha
+</t>
+        </is>
+      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Notes:</t>

</xml_diff>

<commit_message>
Updated the harvesting button to include conditions!
</commit_message>
<xml_diff>
--- a/CrystalDex_Library.xlsx
+++ b/CrystalDex_Library.xlsx
@@ -21196,7 +21196,7 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">07-01-2025, Crystal Screen, DARPin, 1, 1, 1, 1TEL, </t>
+          <t xml:space="preserve">07-01-2025, Crystal_Screen__CS, DARPin, 1, 1, 1, 1TEL, </t>
         </is>
       </c>
     </row>
@@ -21230,7 +21230,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Crystal Screen</t>
+          <t>Crystal_Screen__CS</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -21435,7 +21435,7 @@
       </c>
       <c r="C8" s="22" t="inlineStr">
         <is>
-          <t>1TEL_DARPin_Crystal Screen_A1_top_left_07-01-2025_07-01-2025</t>
+          <t>1TEL_DARPin_Crystal_Screen__CS_A1_top_left_07-01-2025_07-01-2025_harvested</t>
         </is>
       </c>
       <c r="D8" s="3">
@@ -21821,7 +21821,7 @@
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>583x352 um</t>
+          <t>354x354 um</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -22219,7 +22219,7 @@
       </c>
       <c r="C12" s="24" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>L</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -22617,7 +22617,7 @@
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Just a test
+          <t>
 </t>
         </is>
       </c>

</xml_diff>

<commit_message>
You can now export the database to the excel library. Default is to export it every time the program closes. Currently, it overwrites all past data. In the future, I will make it so that only edited trays are overwritten.
</commit_message>
<xml_diff>
--- a/CrystalDex_Library.xlsx
+++ b/CrystalDex_Library.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2Trig-1T-TV-vWa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="04-24-2026_1TEL-GG-UBA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="04-27-2026_1TEL-GG-UBA" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,56 +414,704 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:AC5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>date_set</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>screen</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>top_left_protein_concentration</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>top_right_protein_concentration</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>bottom_left_protein_concentration</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tray ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date Set</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Chaperone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Crystal Screen</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Protein</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Custom Tags</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Top Left Protein Concentration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Top Right Protein Concentration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Bottom Left Protein Concentration</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>06-03-2025</t>
-        </is>
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Crystal_Screen</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>15</v>
-      </c>
-      <c r="D2" t="n">
-        <v>20</v>
-      </c>
-      <c r="E2" t="n">
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tray_id</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>crystal_screen_id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>date_set</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>chaperone</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>crystal_screen</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>custom_tags</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>top_left_protein_concentration</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>top_right_protein_concentration</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>bottom_left_protein_concentration</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>subwell_id</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>subwell_tray_id</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>subwell</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>picture_path</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>conditions</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>minor_axis</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>major_axis</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>number_of_crystals</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>shape</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>possible_salt_crystals</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>precipitation</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>microcrystals</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>glassy_protein_or_artifacts</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>harvester</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>vial_and_run</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>date_snapped</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>10</v>
+      </c>
+      <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>top_left</t>
+        </is>
+      </c>
+      <c r="P5">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_H3_top_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>B12 0.2 M Sodium chloride 0.1 M Tris pH 7.0 35 % v/v (+/-)-2-Methyl-2,4-pentanediol</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>343</v>
+      </c>
+      <c r="S5" t="n">
+        <v>398</v>
+      </c>
+      <c r="T5" t="n">
+        <v>2</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tray ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Date Set</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Chaperone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Crystal Screen</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Protein</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Custom Tags</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Top Left Protein Concentration</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Top Right Protein Concentration</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Bottom Left Protein Concentration</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>04-27-2026</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tray_id</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>crystal_screen_id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>date_set</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>chaperone</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>crystal_screen</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>protein</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>custom_tags</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>top_left_protein_concentration</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>top_right_protein_concentration</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>bottom_left_protein_concentration</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>subwell_id</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>subwell_tray_id</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>subwell</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>picture_path</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>conditions</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>minor_axis</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>major_axis</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>number_of_crystals</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>shape</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>possible_salt_crystals</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>precipitation</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>microcrystals</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>glassy_protein_or_artifacts</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>harvester</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>vial_and_run</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>date_snapped</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04-27-2026</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" t="n">
+        <v>25</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>top_left</t>
+        </is>
+      </c>
+      <c r="P5">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\25_A1_top_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>A1 0.1 M CHES pH 9.5 20 % w/v Polyethylene glycol 8,000</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>176</v>
+      </c>
+      <c r="S5" t="n">
+        <v>92</v>
+      </c>
+      <c r="T5" t="n">
+        <v>1</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>04-27-2026</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed filtering function and harvesting function.
</commit_message>
<xml_diff>
--- a/CrystalDex_Library.xlsx
+++ b/CrystalDex_Library.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -757,6 +757,594 @@
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>2</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>top_right</t>
+        </is>
+      </c>
+      <c r="P6">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_B2_top_right.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>A10 0.1 M Tris pH 7.0 20 % w/v Polyethylene glycol monomethyl ether 2,000</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>205</v>
+      </c>
+      <c r="S6" t="n">
+        <v>267</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>bottom_left</t>
+        </is>
+      </c>
+      <c r="P7">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_A3_bottom_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>B5 0.2 M Lithium sulfate monohydrate 0.1 M Sodium acetate trihydrate pH 4.5 30 % w/v Polyethylene glycol 8,000</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>280</v>
+      </c>
+      <c r="S7" t="n">
+        <v>301</v>
+      </c>
+      <c r="T7" t="n">
+        <v>4</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Miles Bradford</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" t="n">
+        <v>7</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>top_left</t>
+        </is>
+      </c>
+      <c r="P8">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_D2_top_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>A12 0.2 M Calcium acetate hydrate 0.1 M Imidazole pH 8.0 20 % w/v Polyethylene glycol 1,000</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>206</v>
+      </c>
+      <c r="S8" t="n">
+        <v>236</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Miles Bradford</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>10</v>
+      </c>
+      <c r="K9" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>top_left</t>
+        </is>
+      </c>
+      <c r="P9">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_A6_top_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>D5 0.1 M CHES pH 9.5 30 % w/v Polyethylene glycol 3,000</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>223</v>
+      </c>
+      <c r="S9" t="n">
+        <v>476</v>
+      </c>
+      <c r="T9" t="n">
+        <v>6</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Miles Bradford</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>04-24-2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1TEL</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Wizard Screen</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1TEL-GG-UBA</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>10</v>
+      </c>
+      <c r="K10" t="n">
+        <v>9</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>5</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>top_left</t>
+        </is>
+      </c>
+      <c r="P10">
+        <f>HYPERLINK("c:\Users\milesjb\Documents\CrystalDex\Resources\Crystal_Pictures\1_F5_top_left.jpg", "Open Image")</f>
+        <v/>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>D2 0.2 M Lithium sulfate monohydrate 0.1 M CHES pH 9.5 1.0 M Potassium sodium tartrate tetrahydrate</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>367</v>
+      </c>
+      <c r="S10" t="n">
+        <v>377</v>
+      </c>
+      <c r="T10" t="n">
+        <v>5</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Miles Bradford</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>5:22</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>04-28-2026</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Five</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>